<commit_message>
feat: add ASSOCHAM Fintech Festival 2026 and support year/organization metadata
</commit_message>
<xml_diff>
--- a/Google drive links updated.xlsx
+++ b/Google drive links updated.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -971,9 +971,20 @@
         <v>noida, noida office, noida inauguration, office inauguration, office opening, ribbon cutting, grand opening, launch event, office ceremony, branch opening, highspring, highspring noida, highspring inauguration, leadership visit, executives, CEO, management, corporate event, office celebration, employees, event photos, event videos, workplace, office memories, business expansion, opening event, corporate photography, office launch, company event, noida branch</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>ASSOCHAM Fintech Festival 2026</v>
+      </c>
+      <c r="B53" t="str">
+        <v>https://drive.google.com/drive/folders/1e0XhARaCyECfOEPD-aol8NjZgwInkSN-?usp=drive_link</v>
+      </c>
+      <c r="C53" t="str">
+        <v>ASSOCHAM, ASSOCHAM Fintech Festival, ASSOCHAM Fintech Festival 2026, Fintech Festival, FinTech Festival 2026, India International Fintech Festival, India International FinTech Festival 2026, 3rd India International Fintech Festival, 3rd India International FinTech Festival 2026, Fintech, FinTech, Finance, Financial Technology, Digital Finance, Digital Payments, Financial Innovation, Fintech India, India Fintech, Fintech Ecosystem, Financial Services, Banking, Digital Banking, Payments, Innovation, Economic Growth, New Delhi, Delhi, August 2026, 6 August 2026, 7 August 2026, Event, Conference, Festival, Industry Event, Business Event, Photos, Videos, Event Photos, Event Videos, Festival Photos, Festival Videos, ASSOCHAM Event, ASSOCHAM Photos, ASSOCHAM Videos</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C53"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>